<commit_message>
make a final analysis that works on "cereals"
</commit_message>
<xml_diff>
--- a/DataMaster.xlsx
+++ b/DataMaster.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\young\Dropbox\Michael\Work-Uni-Coding\Youngs Farm Analysis\FOG\Work\R&amp;D\Stirlings to Coast\RiskWise\Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DE20ADB-0E83-423F-AFDC-E8E3254FD922}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94E19A01-BD38-45C2-B0FB-35E87A231F56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28950" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{10EDD844-9EC5-4F2C-A4A7-506A3C8B05B2}"/>
+    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{10EDD844-9EC5-4F2C-A4A7-506A3C8B05B2}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -26309,7 +26309,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3321" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3327" uniqueCount="39">
   <si>
     <t>Year</t>
   </si>
@@ -41071,6 +41071,9 @@
       <c r="Q203">
         <v>10</v>
       </c>
+      <c r="R203" t="s">
+        <v>36</v>
+      </c>
       <c r="Y203">
         <v>50</v>
       </c>
@@ -41124,6 +41127,9 @@
       <c r="Q204">
         <v>75.2</v>
       </c>
+      <c r="R204" t="s">
+        <v>36</v>
+      </c>
       <c r="Y204">
         <v>148.9</v>
       </c>
@@ -41177,6 +41183,9 @@
       <c r="Q205">
         <v>175.2</v>
       </c>
+      <c r="R205" t="s">
+        <v>36</v>
+      </c>
       <c r="Y205">
         <v>93.8</v>
       </c>
@@ -43448,7 +43457,7 @@
         <v>79.2</v>
       </c>
       <c r="R239">
-        <v>4.2893586005830899</v>
+        <v>4.5151143164032534</v>
       </c>
       <c r="S239">
         <v>9</v>
@@ -43519,7 +43528,7 @@
         <v>146.19999999999999</v>
       </c>
       <c r="R240">
-        <v>4.0174927113702621</v>
+        <v>4.2289396961792232</v>
       </c>
       <c r="S240">
         <v>10.1</v>
@@ -43590,7 +43599,7 @@
         <v>10</v>
       </c>
       <c r="R241">
-        <v>2.4395043731778423</v>
+        <v>2.710560414642047</v>
       </c>
       <c r="S241">
         <v>8.4</v>
@@ -44078,7 +44087,7 @@
         <v>146.19999999999999</v>
       </c>
       <c r="R248">
-        <v>3.862857142857143</v>
+        <v>4.0661654135338345</v>
       </c>
       <c r="S248">
         <v>10.3</v>
@@ -44149,7 +44158,7 @@
         <v>10</v>
       </c>
       <c r="R249">
-        <v>2.6507142857142858</v>
+        <v>2.9452380952380954</v>
       </c>
       <c r="S249">
         <v>8.3000000000000007</v>
@@ -44220,7 +44229,7 @@
         <v>79.2</v>
       </c>
       <c r="R250">
-        <v>3.3671428571428574</v>
+        <v>3.7412698412698422</v>
       </c>
       <c r="S250">
         <v>9.1</v>
@@ -44495,7 +44504,7 @@
         <v>146.19999999999999</v>
       </c>
       <c r="R254">
-        <v>3.9071428571428566</v>
+        <v>4.3412698412698409</v>
       </c>
       <c r="S254">
         <v>10.3</v>
@@ -44566,7 +44575,7 @@
         <v>79.2</v>
       </c>
       <c r="R255">
-        <v>3.6928571428571426</v>
+        <v>4.1031746031746028</v>
       </c>
       <c r="S255">
         <v>9.5</v>
@@ -44637,7 +44646,7 @@
         <v>10</v>
       </c>
       <c r="R256">
-        <v>1.9728571428571429</v>
+        <v>2.1920634920634923</v>
       </c>
       <c r="S256">
         <v>8.5</v>
@@ -44708,7 +44717,7 @@
         <v>146.19999999999999</v>
       </c>
       <c r="R257">
-        <v>5.3764285714285718</v>
+        <v>5.6593984962406019</v>
       </c>
       <c r="S257">
         <v>10.199999999999999</v>
@@ -44779,7 +44788,7 @@
         <v>10</v>
       </c>
       <c r="R258">
-        <v>3.1678571428571427</v>
+        <v>3.3345864661654137</v>
       </c>
       <c r="S258">
         <v>8</v>
@@ -44850,7 +44859,7 @@
         <v>79.2</v>
       </c>
       <c r="R259">
-        <v>4.7571428571428571</v>
+        <v>5.0075187969924819</v>
       </c>
       <c r="S259">
         <v>9.1999999999999993</v>
@@ -44921,7 +44930,7 @@
         <v>10</v>
       </c>
       <c r="R260">
-        <v>1.357142857142857</v>
+        <v>1.5079365079365079</v>
       </c>
       <c r="S260">
         <v>9.6999999999999993</v>
@@ -44992,7 +45001,7 @@
         <v>79.2</v>
       </c>
       <c r="R261">
-        <v>1.6578571428571429</v>
+        <v>2.0723214285714286</v>
       </c>
       <c r="S261">
         <v>9.5</v>
@@ -45063,7 +45072,7 @@
         <v>146.19999999999999</v>
       </c>
       <c r="R262">
-        <v>2.092857142857143</v>
+        <v>2.46218487394958</v>
       </c>
       <c r="S262">
         <v>10.199999999999999</v>
@@ -45133,6 +45142,9 @@
       <c r="Q263">
         <v>75.2</v>
       </c>
+      <c r="R263" t="s">
+        <v>36</v>
+      </c>
       <c r="Y263">
         <v>67.900000000000006</v>
       </c>
@@ -45186,6 +45198,9 @@
       <c r="Q264">
         <v>175.2</v>
       </c>
+      <c r="R264" t="s">
+        <v>36</v>
+      </c>
       <c r="Y264">
         <v>100.05</v>
       </c>
@@ -45239,6 +45254,9 @@
       <c r="Q265">
         <v>10</v>
       </c>
+      <c r="R265" t="s">
+        <v>36</v>
+      </c>
       <c r="Y265">
         <v>39.9</v>
       </c>
@@ -45293,7 +45311,7 @@
         <v>10</v>
       </c>
       <c r="R266">
-        <v>2.0807142857142855</v>
+        <v>2.6008928571428571</v>
       </c>
       <c r="U266">
         <v>0</v>
@@ -45358,7 +45376,7 @@
         <v>10</v>
       </c>
       <c r="R267">
-        <v>2.6428571428571428</v>
+        <v>2.9365079365079367</v>
       </c>
       <c r="U267">
         <v>0</v>
@@ -45423,7 +45441,7 @@
         <v>10</v>
       </c>
       <c r="R268">
-        <v>2.2164285714285716</v>
+        <v>4.4328571428571433</v>
       </c>
       <c r="U268">
         <v>0</v>
@@ -45488,7 +45506,7 @@
         <v>79.2</v>
       </c>
       <c r="R269">
-        <v>3.2208454810495626</v>
+        <v>3.5787172011661799</v>
       </c>
       <c r="S269">
         <v>9.6</v>
@@ -45559,7 +45577,7 @@
         <v>146.19999999999999</v>
       </c>
       <c r="R270">
-        <v>2.629008746355685</v>
+        <v>3.5053449951409137</v>
       </c>
       <c r="S270">
         <v>10.7</v>
@@ -45630,7 +45648,7 @@
         <v>10</v>
       </c>
       <c r="R271">
-        <v>1.1413994169096211</v>
+        <v>2.2827988338192422</v>
       </c>
       <c r="S271">
         <v>9</v>

</xml_diff>